<commit_message>
MTO Phase 1: template library + per-project versioning + heuristic auto-map with human review
</commit_message>
<xml_diff>
--- a/e2e/sample-mto.xlsx
+++ b/e2e/sample-mto.xlsx
@@ -397,23 +397,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Item</v>
+        <v>Part #</v>
       </c>
       <c r="B1" t="str">
-        <v>Description</v>
+        <v>Desc</v>
       </c>
       <c r="C1" t="str">
         <v>Qty</v>
       </c>
       <c r="D1" t="str">
-        <v>Unit</v>
+        <v>UOM</v>
       </c>
       <c r="E1" t="str">
-        <v>Unit Price</v>
+        <v>Unit Cost</v>
       </c>
       <c r="F1" t="str">
         <v>Total</v>
@@ -479,9 +479,29 @@
         <v>592</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>MULCH-2</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Shredded Hardwood Mulch</v>
+      </c>
+      <c r="C5">
+        <v>60</v>
+      </c>
+      <c r="D5" t="str">
+        <v>CY</v>
+      </c>
+      <c r="E5">
+        <v>42</v>
+      </c>
+      <c r="F5">
+        <v>2520</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>